<commit_message>
15 June 11pm Changes
</commit_message>
<xml_diff>
--- a/attached_assets/charity_full_100_zero_generic_rows_1774031354959.xlsx
+++ b/attached_assets/charity_full_100_zero_generic_rows_1774031354959.xlsx
@@ -5529,9 +5529,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002F923C344106414583D3653D0D956925" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f2c4e54d675ea96885e3b88a53057c94">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca28b9b3-f2c5-4d50-9238-11d2dda0231d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3065d4bc82b8adb8f11be46904ee9fe3" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002F923C344106414583D3653D0D956925" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dcf527ab7ae427f913910ac9968c0a2c">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca28b9b3-f2c5-4d50-9238-11d2dda0231d" xmlns:ns3="b633e036-a69d-499c-b340-accde91e9815" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="058bcd7d7bcd05f14745fd7c7f7f8d3f" ns2:_="" ns3:_="">
     <xsd:import namespace="ca28b9b3-f2c5-4d50-9238-11d2dda0231d"/>
+    <xsd:import namespace="b633e036-a69d-499c-b340-accde91e9815"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -5541,6 +5542,12 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5565,6 +5572,50 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="44f85279-4518-4657-99cc-613eccc5bd09" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b633e036-a69d-499c-b340-accde91e9815" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{04c15fe6-ae9b-4a82-b06f-b0baf4d2d5ea}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="b633e036-a69d-499c-b340-accde91e9815">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -5677,12 +5728,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="b633e036-a69d-499c-b340-accde91e9815" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca28b9b3-f2c5-4d50-9238-11d2dda0231d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE3681E-DD9C-4D77-B652-505B6334148D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CDEBD0D-6A3D-4BB2-9306-C62DCA66C30A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>